<commit_message>
fix: store super hide as an option
- Move super_hide from the user row to the option table
- Toggle super hide through the in-game option API instead of a full save
- Hide super-hidden characters from name2ch lookups by players
- Count receiver escrow when giving bundled items
- Return items that do not fit back to the giver or trader
- Subtract only offered counts when checking trade capacity
</commit_message>
<xml_diff>
--- a/resources/table/enum.xlsx
+++ b/resources/table/enum.xlsx
@@ -1,35 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="600" firstSheet="14" activeTab="23" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="GENDER" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ROLE" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="DIRECTION" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DESTROY_TYPE" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="OBJECT_TYPE" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="DIALOG_RESULT" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="DIVINE_BEAST" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="NATION" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ACTION" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="STATE" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="CROWD_CONTROL" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="SOUND" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="DURATION" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="UPDATE_STATE_LEVEL" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="CARDINAL_DIRECTION" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="BROADCAST_TYPE" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="OPTION" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="MESSAGE_TYPE" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="SWAP_TYPE" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="CHAT_TYPE" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="WEATHER_TYPE" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="TIMER_TYPE" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="HEAD_MARKER" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="INSTANCE_RULE_TYPE" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GENDER" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROLE" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DIRECTION" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DESTROY_TYPE" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OBJECT_TYPE" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DIALOG_RESULT" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DIVINE_BEAST" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NATION" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACTION" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STATE" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CROWD_CONTROL" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOUND" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DURATION" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UPDATE_STATE_LEVEL" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CARDINAL_DIRECTION" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BROADCAST_TYPE" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPTION" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MESSAGE_TYPE" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SWAP_TYPE" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHAT_TYPE" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WEATHER_TYPE" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TIMER_TYPE" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HEAD_MARKER" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTANCE_RULE_TYPE" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="181029" fullCalcOnLoad="1"/>
@@ -1134,7 +1134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15.25" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -1310,6 +1310,18 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SUPER_HIDE</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0x80</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1692,12 +1704,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>0x03</t>
         </is>

</xml_diff>